<commit_message>
Correct AS-c.3.1.2 genotype name to AS-c.3.1.1
</commit_message>
<xml_diff>
--- a/dependencies/genotype_key_asia.xlsx
+++ b/dependencies/genotype_key_asia.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R88dd3f3fe2bd4419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R08ef4d37cdff4d49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3604,7 +3604,7 @@
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="str">
-        <x:v>AS-c.3.1.2</x:v>
+        <x:v>AS-c.3.1.1</x:v>
       </x:c>
       <x:c r="B116" t="str">
         <x:v>PB2_group81</x:v>

</xml_diff>